<commit_message>
Tablas_Stock archivo v2 - Ago-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_08.xlsx
+++ b/Tablas/Tablas_Stock_2026_08.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 89% sobre 565 incidentes; 'Luminaria superior e inferior apagada du' lidera con 398 casos (91% cierre). Gestion interna 50%.</t>
+          <t>El área que mejor responde: cierra el 89% de sus 565 reclamos en 4 días promedio. Siete de cada diez son luminarias apagadas de noche (398 casos), una suba que se repite cada invierno. La mitad de su carga la detecta el propio municipio, no el vecino.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre bajo 49% sobre 98 incidentes; 'Inconvenientes con intervenciones de arb' lidera con 33 casos (88% cierre). SLA 77%, sat 54%.</t>
+          <t>Más que duplicó su demanda (98 casos) y el cierre cayó a 49%: resuelve rápido lo que atiende, pero deja la mitad sin cerrar. El corte de césped arrancó un mes antes que el año pasado y ya acumula 23 reclamos con apenas 17% de cierre.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre bajo 20% sobre 405 incidentes; 'Bache en calle de asfalto' lidera con 178 casos (19% cierre). Dias prom 9.0 elevado.</t>
+          <t>El cuadro más crítico del municipio: recibe el máximo histórico de reclamos (405, el doble que en enero) y cierra uno de cada cinco, con 9 días promedio. Los baches de asfalto (178 casos) marcan un deterioro real del pavimento, no estacional.</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 78% sobre 101 incidentes; 'Falta de Habilitación - Actividad no dec' lidera con 37 casos (89% cierre). SLA 52%, sat 33%.</t>
+          <t>Cierra bien —78% de 101 reclamos— pero el vecino no lo percibe así: la satisfacción es del 33%, la más baja del municipio. Predominan las denuncias por falta de habilitación comercial (37 casos), donde cerrar el expediente no siempre resuelve el problema.</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre moderado 55% sobre 275 incidentes; 'Cable cortado' lidera con 77 casos (12% cierre). SLA 76%, sat 47%.</t>
+          <t>Demanda en baja sostenida (275 casos, desde 393 en enero), pero con el cierre partido en dos: resuelve el 100% de las desratizaciones y apenas el 12% de los cables cortados y el 22% de los postes en mal estado.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 86% sobre 1657 incidentes; 'Retiro de escombros y/o restos de obra' lidera con 468 casos (91% cierre). SLA 50%, sat 73%.</t>
+          <t>Concentra casi la mitad de la demanda del municipio (1.657 casos) y la viene reduciendo con fuerza: 45% menos que en enero. Cierra el 86% en 5 días. El grueso son retiros a domicilio de escombros, restos de poda y objetos en desuso.</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 70% sobre 458 incidentes; 'Vehículos Abandonados' lidera con 346 casos (76% cierre). Sat 71% (muestra insuficiente).</t>
+          <t>Demanda estable (458 casos) y cierre del 70%, pero lento: solo el 31% se resuelve dentro del plazo comprometido. Tres de cada cuatro reclamos son vehículos abandonados (346 casos). La satisfacción del 71% surge de apenas 17 respuestas.</t>
         </is>
       </c>
     </row>

</xml_diff>